<commit_message>
fixed changes pop out
</commit_message>
<xml_diff>
--- a/schedule/2026_datascience_organization.xlsx
+++ b/schedule/2026_datascience_organization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wlperry/Documents/r_projects/web_datascience_website_2026/schedule/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D720715-479F-D447-88C5-55B24FBB2E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89483890-0802-B549-9C04-476B3CB2389A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35300" yWindow="-2740" windowWidth="22220" windowHeight="19640" xr2:uid="{85A1AE42-D6B2-9944-9D18-E3A7EC306998}"/>
+    <workbookView xWindow="35700" yWindow="-8840" windowWidth="20980" windowHeight="27200" xr2:uid="{85A1AE42-D6B2-9944-9D18-E3A7EC306998}"/>
   </bookViews>
   <sheets>
     <sheet name="schedule" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="59">
   <si>
     <t>Week</t>
   </si>
@@ -66,10 +66,13 @@
     <t>Points</t>
   </si>
   <si>
+    <t>Final Project</t>
+  </si>
+  <si>
     <t>Total</t>
   </si>
   <si>
-    <t>add in mst suprising thing at the end… only grade that.</t>
+    <t>Project Pitch</t>
   </si>
   <si>
     <t>Project design and graphing</t>
@@ -145,6 +148,72 @@
   </si>
   <si>
     <t>Quiuzzes</t>
+  </si>
+  <si>
+    <t>Intro and data</t>
+  </si>
+  <si>
+    <t>GGPlot</t>
+  </si>
+  <si>
+    <t>wrangling</t>
+  </si>
+  <si>
+    <t>Quarto Markdown</t>
+  </si>
+  <si>
+    <t>T Tests</t>
+  </si>
+  <si>
+    <t>Weather Data</t>
+  </si>
+  <si>
+    <t>Anova</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lake Superior Ice </t>
+  </si>
+  <si>
+    <t>Joins</t>
+  </si>
+  <si>
+    <t>Final Projects</t>
+  </si>
+  <si>
+    <t>Working on Final Projects - Help sessions</t>
+  </si>
+  <si>
+    <t>Quiz 1</t>
+  </si>
+  <si>
+    <t>Quiz 2</t>
+  </si>
+  <si>
+    <t>Quiz 3</t>
+  </si>
+  <si>
+    <t>Quiz 4</t>
+  </si>
+  <si>
+    <t>Quiz 5</t>
+  </si>
+  <si>
+    <t>Quiz 6</t>
+  </si>
+  <si>
+    <t>Quiz 7</t>
+  </si>
+  <si>
+    <t>Quiz 8</t>
+  </si>
+  <si>
+    <t>Quiz 9</t>
+  </si>
+  <si>
+    <t>Quizzes (10 pts each)</t>
+  </si>
+  <si>
+    <t>Project design - graphing</t>
   </si>
 </sst>
 </file>
@@ -154,7 +223,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -168,6 +237,11 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="ArialMT"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="ArialMT"/>
@@ -187,7 +261,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -210,92 +284,37 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -630,690 +649,784 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01800ABB-550A-EE4C-B9D4-F43DE81AFA49}">
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="49.7109375" customWidth="1"/>
-    <col min="10" max="10" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17" thickBot="1">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" s="5" t="s">
+      <c r="F1" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="5" t="s">
-        <v>8</v>
+      <c r="J1" s="11" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="10">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="11">
+      <c r="B2" s="3">
         <v>46266</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2">
-        <v>20</v>
+      <c r="C2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="I2" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="J2" s="6">
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="10">
+      <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="3">
         <f>B2+2</f>
         <v>46268</v>
       </c>
-      <c r="C3" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2">
+      <c r="C3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="I3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" s="6">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="10">
+      <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="3">
         <f>B3+5</f>
         <v>46273</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2">
+        <v>17</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J4" s="6">
         <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="10">
+      <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="3">
         <f>B4+2</f>
         <v>46275</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2">
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="I5" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" s="6">
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="10">
+      <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="3">
         <f>B5+5</f>
         <v>46280</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="I6" s="6"/>
+        <v>19</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="J6" s="6">
         <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="10">
+      <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="3">
         <f>B6+2</f>
         <v>46282</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2">
         <v>20</v>
       </c>
+      <c r="E7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="I7" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="J7" s="6">
+        <v>20</v>
+      </c>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="10">
+      <c r="A8" s="2">
         <v>4</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="3">
         <f>B7+5</f>
         <v>46287</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3">
-        <v>35</v>
+        <v>21</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="6">
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="10">
+      <c r="A9" s="2">
         <v>4</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="3">
         <f>B8+2</f>
         <v>46289</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2">
-        <v>15</v>
+        <v>22</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="I9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J9" s="6">
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="10">
-        <v>5</v>
-      </c>
-      <c r="B10" s="11">
+      <c r="A10" s="2">
+        <v>5</v>
+      </c>
+      <c r="B10" s="3">
         <f>B9+5</f>
         <v>46294</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="2">
+        <v>23</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="I10" s="6">
         <v>20</v>
       </c>
+      <c r="J10" s="6">
+        <v>30</v>
+      </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="10">
-        <v>5</v>
-      </c>
-      <c r="B11" s="11">
+      <c r="A11" s="2">
+        <v>5</v>
+      </c>
+      <c r="B11" s="3">
         <f>B10+2</f>
         <v>46296</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2">
-        <v>15</v>
+        <v>24</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="I11" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="J11" s="9">
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="10">
-        <v>6</v>
-      </c>
-      <c r="B12" s="11">
+      <c r="A12" s="2">
+        <v>6</v>
+      </c>
+      <c r="B12" s="3">
         <f>B11+5</f>
         <v>46301</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="2">
         <v>25</v>
       </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J12" s="9">
+        <v>20</v>
+      </c>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="10">
-        <v>6</v>
-      </c>
-      <c r="B13" s="11">
+      <c r="A13" s="2">
+        <v>6</v>
+      </c>
+      <c r="B13" s="3">
         <f>B12+2</f>
         <v>46303</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2">
-        <v>15</v>
+        <v>26</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="2"/>
+      <c r="I13" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="J13" s="9">
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="10">
+      <c r="A14" s="2">
         <v>7</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="3">
         <f>B13+5</f>
         <v>46308</v>
       </c>
-      <c r="C14" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="2">
-        <v>25</v>
+      <c r="C14" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J14" s="9">
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="15">
         <v>7</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="17">
         <f>B14+2</f>
         <v>46310</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="17" t="s">
         <v>5</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="17"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="10"/>
+      <c r="I15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J15" s="9">
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="15">
         <v>8</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="17">
         <f>B15+5</f>
         <v>46315</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="17" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E16" s="15"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="17"/>
-      <c r="I16" s="7"/>
+      <c r="F16" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G16" s="10"/>
+      <c r="I16" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="J16" s="9">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="17" thickBot="1">
-      <c r="A17" s="18">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" s="16">
         <v>8</v>
       </c>
-      <c r="B17" s="16">
+      <c r="B17" s="17">
         <f>B16+2</f>
         <v>46317</v>
       </c>
-      <c r="C17" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="E17" s="15"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="17"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="5">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
-      <c r="A18" s="18">
+      <c r="C17" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="10"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="9"/>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" s="16">
         <v>9</v>
       </c>
-      <c r="B18" s="16">
+      <c r="B18" s="17">
         <f>B17+5</f>
         <v>46322</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="19" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="17"/>
-      <c r="I18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="10"/>
+      <c r="I18" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="J18" s="6">
+        <f>SUM(J2:J17)</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" s="20">
         <v>9</v>
       </c>
-      <c r="J18" s="4">
-        <f>SUM(J2:J17)</f>
-        <v>360</v>
-      </c>
-      <c r="K18">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11">
-      <c r="A19" s="21">
-        <v>9</v>
-      </c>
-      <c r="B19" s="22">
+      <c r="B19" s="21">
         <f>B18+2</f>
         <v>46324</v>
       </c>
-      <c r="C19" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="17"/>
-    </row>
-    <row r="20" spans="1:11">
+      <c r="C19" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="10"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+    </row>
+    <row r="20" spans="1:10">
       <c r="A20" s="15">
         <v>10</v>
       </c>
-      <c r="B20" s="16">
+      <c r="B20" s="17">
         <f>B19+5</f>
         <v>46329</v>
       </c>
-      <c r="C20" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" t="s">
-        <v>32</v>
-      </c>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="17"/>
-    </row>
-    <row r="21" spans="1:11">
+      <c r="C20" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" s="18"/>
+      <c r="F20" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="G20" s="10"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+    </row>
+    <row r="21" spans="1:10">
       <c r="A21" s="15">
         <v>10</v>
       </c>
-      <c r="B21" s="16">
+      <c r="B21" s="17">
         <f>B20+2</f>
         <v>46331</v>
       </c>
-      <c r="C21" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" t="s">
-        <v>32</v>
-      </c>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="17"/>
-    </row>
-    <row r="22" spans="1:11">
-      <c r="A22" s="10">
+      <c r="C21" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="F21" s="2"/>
+      <c r="G21" s="10"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" s="2">
         <v>11</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="3">
         <f>B21+5</f>
         <v>46336</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="I22" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
-      <c r="A23" s="10">
+        <v>31</v>
+      </c>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" s="2">
         <v>11</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="3">
         <f>B22+2</f>
         <v>46338</v>
       </c>
-      <c r="C23" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="15"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-    </row>
-    <row r="24" spans="1:11">
-      <c r="A24" s="10">
+      <c r="C23" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="18"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" s="2">
         <v>12</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="3">
         <f>B23+5</f>
         <v>46343</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-    </row>
-    <row r="25" spans="1:11">
-      <c r="A25" s="10">
+        <v>32</v>
+      </c>
+      <c r="E24" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="F24" s="15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" s="2">
         <v>12</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="3">
         <f>B24+2</f>
         <v>46345</v>
       </c>
-      <c r="C25" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-    </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="10">
+      <c r="C25" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="2">
         <v>13</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="3">
         <f>B25+5</f>
         <v>46350</v>
       </c>
-      <c r="C26" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-    </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="21">
+      <c r="C26" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="F26" s="22"/>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="20">
         <v>13</v>
       </c>
-      <c r="B27" s="22">
+      <c r="B27" s="21">
         <f>B26+2</f>
         <v>46352</v>
       </c>
-      <c r="C27" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="21" t="s">
+      <c r="C27" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" s="2">
         <v>14</v>
       </c>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
-    </row>
-    <row r="28" spans="1:11">
-      <c r="A28" s="10">
-        <v>14</v>
-      </c>
-      <c r="B28" s="11">
+      <c r="B28" s="3">
         <f>B27+5</f>
         <v>46357</v>
       </c>
-      <c r="C28" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-    </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="10">
+      <c r="C28" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" s="2">
         <v>14</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="3">
         <f>B28+2</f>
         <v>46359</v>
       </c>
-      <c r="C29" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-    </row>
-    <row r="30" spans="1:11">
-      <c r="A30" s="10">
+      <c r="C29" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" s="2">
         <v>15</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="3">
         <f>B29+5</f>
         <v>46364</v>
       </c>
-      <c r="C30" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-    </row>
-    <row r="31" spans="1:11">
-      <c r="A31" s="10">
+      <c r="C30" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="I30" s="6"/>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" s="2">
         <v>15</v>
       </c>
-      <c r="B31" s="11">
+      <c r="B31" s="3">
         <f>B30+2</f>
         <v>46366</v>
       </c>
-      <c r="C31" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="12"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-    </row>
-    <row r="32" spans="1:11">
-      <c r="A32" s="10"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" s="10"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34" s="10"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" s="10"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36" s="10"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" s="10"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" s="10"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="10"/>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" s="10"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="10"/>
+      <c r="C31" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" s="22"/>
+      <c r="I31" s="6"/>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="2"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="I32" s="6"/>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="6"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="I33" s="9"/>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="6"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="I34" s="9"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="6"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="I35" s="6"/>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="6"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="I36" s="9"/>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="6"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="I37" s="12"/>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="6"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+      <c r="I38" s="12"/>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="6"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+      <c r="I39" s="12"/>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="I40" s="13"/>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="I41" s="13"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>